<commit_message>
updated summary statistics and explorations on author info
</commit_message>
<xml_diff>
--- a/analysis/deliverable/reports/summary_statistics_final.xlsx
+++ b/analysis/deliverable/reports/summary_statistics_final.xlsx
@@ -8589,7 +8589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8607,154 +8607,190 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>source_partition</t>
+          <t>clean_metadata.parquet</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Raw TDM metadata partition directory.</t>
+          <t>Cleaned English document metadata export with original TDM fields renamed to snake_case plus parsed dates, publisher geography diagnostics, author counts, term counts, and page counts.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>partition_family</t>
+          <t>metadata_topics_sentiment.parquet</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Partition source family inferred from the export name.</t>
+          <t>Document-level analytical feature export keyed by goid, including normalized titles, canonical publication titles, duplicate flags, NMF topic assignments, and Loughran-McDonald sentiment scores.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>goid</t>
+          <t>source_partition</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TDM document identifier; primary document key.</t>
+          <t>Raw TDM metadata partition directory.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>publication_date</t>
+          <t>partition_family</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Parsed publication date from Date.</t>
+          <t>Partition source family inferred from the export name.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>year</t>
+          <t>goid</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Publication year.</t>
+          <t>TDM document identifier; primary document key.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>decade</t>
+          <t>publication_date</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Publication decade.</t>
+          <t>Parsed publication date from Date.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>publication_title_normalized</t>
+          <t>year</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Normalized publication title for grouping aliases.</t>
+          <t>Publication year.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>publisher_region</t>
+          <t>decade</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Publisher geography diagnostic; not used as the primary sample filter.</t>
+          <t>Publication decade.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>duplicate_normalized_title_date_publication</t>
+          <t>publication_title_canonical</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>True for rows in a duplicate group by normalized title, date, and publication.</t>
+          <t>Conservative canonical publication title built from token-aware alias rules.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>is_conservative_duplicate_extra</t>
+          <t>publication_title_normalized</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>True for rows dropped from the conservative deduplicated export.</t>
+          <t>Normalized publication title for grouping aliases.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>topic_id</t>
+          <t>publisher_region</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NMF topic assigned from Title + Subject Terms + Class Terms.</t>
+          <t>Publisher geography diagnostic; not used as the primary sample filter.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>title_only_topic_id</t>
+          <t>duplicate_normalized_title_date_publication</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sensitivity topic assignment using title text only.</t>
+          <t>True for rows in a duplicate group by normalized title, date, and publication.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>is_conservative_duplicate_extra</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>True for extra rows under the conservative normalized title/date/publication duplicate rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>topic_id</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NMF topic assigned from Title + Subject Terms + Class Terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>title_only_topic_id</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sensitivity topic assignment using title text only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>lm_net_tone</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Loughran-McDonald positive minus negative word count divided by LM token count.</t>
         </is>

</xml_diff>